<commit_message>
made a lot of changes lol
</commit_message>
<xml_diff>
--- a/output/values_2 (version 1) (version 1).xlsx
+++ b/output/values_2 (version 1) (version 1).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eligh\summer\research\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D55D5A8-A033-45AF-9C49-CD55B69DC268}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84AD1D97-B839-4CD8-900E-1369F9A43E9D}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{FA81AE3B-DEFA-473D-BE0F-682341565E4F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="1" activeTab="8" xr2:uid="{FA81AE3B-DEFA-473D-BE0F-682341565E4F}"/>
   </bookViews>
   <sheets>
     <sheet name="q,d_sum" sheetId="9" r:id="rId1"/>
@@ -40,7 +40,6 @@
     <definedName name="totalenergies" localSheetId="4">energies!$A$2:$H$67</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -1171,13 +1170,7 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <numFmt numFmtId="164" formatCode="0.0000000000"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="0.0000000000"/>
@@ -1198,7 +1191,13 @@
       <numFmt numFmtId="164" formatCode="0.0000000000"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="0.0000000000"/>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1365,7 +1364,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{7E5C5FCA-A89A-479C-801D-CAF2AD735CAE}" name="dipoles__3" displayName="dipoles__3" ref="A1:E17" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:E17" xr:uid="{A87FE459-94FB-4F79-91E5-4277EE19594E}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{4CB0D2CF-69C0-4090-9887-17E3635172BA}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{4CB0D2CF-69C0-4090-9887-17E3635172BA}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="12"/>
     <tableColumn id="2" xr3:uid="{F49D68FA-5C32-4A23-B61B-0EA0675B314E}" uniqueName="2" name="X" queryTableFieldId="2"/>
     <tableColumn id="3" xr3:uid="{CD58B8FE-1964-46C1-8D48-7FBF524A8515}" uniqueName="3" name="Y" queryTableFieldId="3"/>
     <tableColumn id="4" xr3:uid="{0C627D5A-60CF-4200-9978-EF5B57267C4C}" uniqueName="4" name="Z" queryTableFieldId="4"/>
@@ -1379,7 +1378,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{99E9D2B2-B032-4DAA-BDCB-532781F5FB2B}" name="quadrupoles__2" displayName="quadrupoles__2" ref="A1:G17" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:G17" xr:uid="{30E8BC04-BAFC-497E-9EAB-0E28B95B0AB7}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{C2439B7F-954F-4A0B-918D-D9592A797649}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{C2439B7F-954F-4A0B-918D-D9592A797649}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="11"/>
     <tableColumn id="2" xr3:uid="{2A405823-68C2-444A-A9F9-85356F1B259D}" uniqueName="2" name="XX" queryTableFieldId="2"/>
     <tableColumn id="3" xr3:uid="{91C1ECBC-1EC6-4813-A8F2-97BCDD61B07F}" uniqueName="3" name="XY" queryTableFieldId="3"/>
     <tableColumn id="4" xr3:uid="{A3727430-7E1F-4F3D-8943-224DCCFA5562}" uniqueName="4" name="YY" queryTableFieldId="4"/>
@@ -1395,14 +1394,14 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4386FDD3-088E-4C5E-ADFA-BA691E95A684}" name="totalenergies" displayName="totalenergies_1" ref="A2:H18" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A2:H18" xr:uid="{8C090970-03C1-41AB-80D8-CA9E61B2B212}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{992DE68D-54AF-4D53-8730-2AD79DC77F6E}" uniqueName="1" name="molecule_method_basis" queryTableFieldId="1" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{EBE0C37B-7FB0-4BCD-BAE6-C2CB32737A1C}" uniqueName="2" name="0 field" queryTableFieldId="2" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{AB431FC4-9849-45BF-A6CD-81755AE22693}" uniqueName="3" name="XX" queryTableFieldId="3" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{6C7DB2F4-CEAD-462B-AC7B-3CEB936CD473}" uniqueName="4" name="-XX" queryTableFieldId="4" dataDxfId="10"/>
-    <tableColumn id="5" xr3:uid="{0EDF1F37-9AB9-4F7E-A5AF-4A4626C08892}" uniqueName="5" name="ZZ" queryTableFieldId="5" dataDxfId="9"/>
-    <tableColumn id="6" xr3:uid="{50E61199-067E-434D-95D3-29835A4275DE}" uniqueName="6" name="-ZZ" queryTableFieldId="6" dataDxfId="8"/>
-    <tableColumn id="7" xr3:uid="{40444CC4-157B-4C0B-AFE0-75FA7D33A7A4}" uniqueName="7" name="Z" queryTableFieldId="7" dataDxfId="7"/>
-    <tableColumn id="8" xr3:uid="{442DFE81-329D-4905-BFF5-766A790A5492}" uniqueName="8" name="-Z" queryTableFieldId="8" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{992DE68D-54AF-4D53-8730-2AD79DC77F6E}" uniqueName="1" name="molecule_method_basis" queryTableFieldId="1" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{EBE0C37B-7FB0-4BCD-BAE6-C2CB32737A1C}" uniqueName="2" name="0 field" queryTableFieldId="2" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{AB431FC4-9849-45BF-A6CD-81755AE22693}" uniqueName="3" name="XX" queryTableFieldId="3" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{6C7DB2F4-CEAD-462B-AC7B-3CEB936CD473}" uniqueName="4" name="-XX" queryTableFieldId="4" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{0EDF1F37-9AB9-4F7E-A5AF-4A4626C08892}" uniqueName="5" name="ZZ" queryTableFieldId="5" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{50E61199-067E-434D-95D3-29835A4275DE}" uniqueName="6" name="-ZZ" queryTableFieldId="6" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{40444CC4-157B-4C0B-AFE0-75FA7D33A7A4}" uniqueName="7" name="Z" queryTableFieldId="7" dataDxfId="4"/>
+    <tableColumn id="8" xr3:uid="{442DFE81-329D-4905-BFF5-766A790A5492}" uniqueName="8" name="-Z" queryTableFieldId="8" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1412,7 +1411,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{0618320E-AAE4-4F4B-934A-BB8779FB9979}" name="ccsdenergies5" displayName="ccsdenergies5" ref="A21:H37" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A21:H37" xr:uid="{CB974A09-2327-46D5-8B7F-548A8B71285B}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{9DD87CA6-5A5B-4DF3-ABE8-1CCD5FFB7653}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{9DD87CA6-5A5B-4DF3-ABE8-1CCD5FFB7653}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="2"/>
     <tableColumn id="2" xr3:uid="{51E1C58B-7ABF-40C4-9EA2-66C736148784}" uniqueName="2" name="Column2" queryTableFieldId="2"/>
     <tableColumn id="3" xr3:uid="{D01990F7-53C9-4305-B7D2-B4DCFDBE279F}" uniqueName="3" name="Column3" queryTableFieldId="3"/>
     <tableColumn id="4" xr3:uid="{47369D86-B10C-453D-A266-A378CCD0D107}" uniqueName="4" name="Column4" queryTableFieldId="4"/>
@@ -1429,7 +1428,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{8D7A3A0E-3282-4FAD-A6EC-3BF5386E63F5}" name="mp2energies" displayName="mp2energies" ref="A40:H56" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A40:H56" xr:uid="{14A6F1F6-7465-4A11-91AC-1939E0374CDF}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{44B6C42B-467A-4228-A032-7FE101BC31EF}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{44B6C42B-467A-4228-A032-7FE101BC31EF}" uniqueName="1" name="Column1" queryTableFieldId="1" dataDxfId="1"/>
     <tableColumn id="2" xr3:uid="{AA45125D-48A8-439F-B2CC-C7D41C6FE06E}" uniqueName="2" name="Column2" queryTableFieldId="2"/>
     <tableColumn id="3" xr3:uid="{E49277FB-9650-492B-842C-40CD91D0552C}" uniqueName="3" name="Column3" queryTableFieldId="3"/>
     <tableColumn id="4" xr3:uid="{13E9BC6F-5A77-4854-B402-88311A68C480}" uniqueName="4" name="Column4" queryTableFieldId="4"/>

</xml_diff>